<commit_message>
added units to new GDP field
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/sfdr/sfdr.xlsx
+++ b/dataland-framework-toolbox/inputs/sfdr/sfdr.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d93912\IdeaProjects\Dataland\dataland-framework-toolbox\inputs\sfdr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDDF7F7-2707-4710-B87B-DE2E1C34A602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81786C1F-2A5F-471C-8D4E-E5E710325A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="388">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -1303,6 +1303,9 @@
   </si>
   <si>
     <t>A country’s total economic output in euros. See also Regulation (EU) 2022/1288, Annex I, formula (4). Linked to Regulation (EU) 2022/1288, Annex I, Table 1, Adverse sustainability indicator 15</t>
+  </si>
+  <si>
+    <t>USD</t>
   </si>
 </sst>
 </file>
@@ -1410,7 +1413,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1464,7 +1467,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -1853,7 +1855,7 @@
       </c>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="23">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -1887,13 +1889,13 @@
       <c r="N2" s="6"/>
     </row>
     <row r="3" spans="1:18">
-      <c r="A3" s="23">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="23" t="s">
         <v>25</v>
       </c>
       <c r="D3" s="8" t="s">
@@ -2058,10 +2060,18 @@
         <v>385</v>
       </c>
       <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
+      <c r="H7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>20</v>
+      </c>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
       <c r="N7" s="12"/>
@@ -2345,7 +2355,7 @@
       <c r="R14" s="12"/>
     </row>
     <row r="15" spans="1:18" s="6" customFormat="1">
-      <c r="A15" s="23">
+      <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -2378,7 +2388,7 @@
       </c>
     </row>
     <row r="16" spans="1:18" s="6" customFormat="1">
-      <c r="A16" s="23">
+      <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -2409,7 +2419,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" s="6" customFormat="1">
-      <c r="A17" s="23">
+      <c r="A17" s="4">
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -2442,7 +2452,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" s="6" customFormat="1">
-      <c r="A18" s="23">
+      <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -2475,7 +2485,7 @@
       </c>
     </row>
     <row r="19" spans="1:11" s="6" customFormat="1">
-      <c r="A19" s="23">
+      <c r="A19" s="4">
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
@@ -2506,7 +2516,7 @@
       </c>
     </row>
     <row r="20" spans="1:11" s="6" customFormat="1">
-      <c r="A20" s="23">
+      <c r="A20" s="4">
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -2537,7 +2547,7 @@
       </c>
     </row>
     <row r="21" spans="1:11" s="6" customFormat="1">
-      <c r="A21" s="23">
+      <c r="A21" s="4">
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
@@ -2568,7 +2578,7 @@
       </c>
     </row>
     <row r="22" spans="1:11" s="6" customFormat="1">
-      <c r="A22" s="23">
+      <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -2601,7 +2611,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" s="6" customFormat="1">
-      <c r="A23" s="23">
+      <c r="A23" s="4">
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
@@ -2632,7 +2642,7 @@
       </c>
     </row>
     <row r="24" spans="1:11" s="6" customFormat="1">
-      <c r="A24" s="23">
+      <c r="A24" s="4">
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -2663,7 +2673,7 @@
       </c>
     </row>
     <row r="25" spans="1:11" s="6" customFormat="1">
-      <c r="A25" s="23">
+      <c r="A25" s="4">
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
@@ -2694,7 +2704,7 @@
       </c>
     </row>
     <row r="26" spans="1:11" s="6" customFormat="1">
-      <c r="A26" s="23">
+      <c r="A26" s="4">
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
@@ -2725,7 +2735,7 @@
       </c>
     </row>
     <row r="27" spans="1:11" s="6" customFormat="1">
-      <c r="A27" s="23">
+      <c r="A27" s="4">
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
@@ -2756,7 +2766,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" s="6" customFormat="1">
-      <c r="A28" s="23">
+      <c r="A28" s="4">
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
@@ -2787,7 +2797,7 @@
       </c>
     </row>
     <row r="29" spans="1:11" s="6" customFormat="1">
-      <c r="A29" s="23">
+      <c r="A29" s="4">
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
@@ -2818,7 +2828,7 @@
       </c>
     </row>
     <row r="30" spans="1:11" s="6" customFormat="1">
-      <c r="A30" s="23">
+      <c r="A30" s="4">
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
@@ -2849,7 +2859,7 @@
       </c>
     </row>
     <row r="31" spans="1:11" s="6" customFormat="1">
-      <c r="A31" s="23">
+      <c r="A31" s="4">
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
@@ -2880,7 +2890,7 @@
       </c>
     </row>
     <row r="32" spans="1:11" s="6" customFormat="1">
-      <c r="A32" s="23">
+      <c r="A32" s="4">
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
@@ -2911,7 +2921,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" s="6" customFormat="1">
-      <c r="A33" s="23">
+      <c r="A33" s="4">
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
@@ -2941,7 +2951,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" s="6" customFormat="1">
-      <c r="A34" s="23">
+      <c r="A34" s="4">
         <v>33</v>
       </c>
       <c r="B34" s="7" t="s">
@@ -2972,7 +2982,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" s="6" customFormat="1">
-      <c r="A35" s="23">
+      <c r="A35" s="4">
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
@@ -3003,7 +3013,7 @@
       </c>
     </row>
     <row r="36" spans="1:11" s="6" customFormat="1">
-      <c r="A36" s="23">
+      <c r="A36" s="4">
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
@@ -3036,7 +3046,7 @@
       </c>
     </row>
     <row r="37" spans="1:11" s="6" customFormat="1">
-      <c r="A37" s="23">
+      <c r="A37" s="4">
         <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
@@ -3069,7 +3079,7 @@
       </c>
     </row>
     <row r="38" spans="1:11" s="6" customFormat="1">
-      <c r="A38" s="23">
+      <c r="A38" s="4">
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -3102,7 +3112,7 @@
       </c>
     </row>
     <row r="39" spans="1:11" s="6" customFormat="1">
-      <c r="A39" s="23">
+      <c r="A39" s="4">
         <v>38</v>
       </c>
       <c r="B39" s="4" t="s">
@@ -3135,7 +3145,7 @@
       </c>
     </row>
     <row r="40" spans="1:11" s="6" customFormat="1">
-      <c r="A40" s="23">
+      <c r="A40" s="4">
         <v>39</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -3168,7 +3178,7 @@
       </c>
     </row>
     <row r="41" spans="1:11" s="6" customFormat="1">
-      <c r="A41" s="23">
+      <c r="A41" s="4">
         <v>40</v>
       </c>
       <c r="B41" s="4" t="s">
@@ -3201,7 +3211,7 @@
       </c>
     </row>
     <row r="42" spans="1:11" s="6" customFormat="1">
-      <c r="A42" s="23">
+      <c r="A42" s="4">
         <v>41</v>
       </c>
       <c r="B42" s="4" t="s">
@@ -3234,7 +3244,7 @@
       </c>
     </row>
     <row r="43" spans="1:11" s="6" customFormat="1">
-      <c r="A43" s="23">
+      <c r="A43" s="4">
         <v>42</v>
       </c>
       <c r="B43" s="4" t="s">
@@ -3267,7 +3277,7 @@
       </c>
     </row>
     <row r="44" spans="1:11" s="6" customFormat="1">
-      <c r="A44" s="23">
+      <c r="A44" s="4">
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -3300,7 +3310,7 @@
       </c>
     </row>
     <row r="45" spans="1:11" s="6" customFormat="1">
-      <c r="A45" s="23">
+      <c r="A45" s="4">
         <v>44</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -3333,7 +3343,7 @@
       </c>
     </row>
     <row r="46" spans="1:11" s="6" customFormat="1">
-      <c r="A46" s="23">
+      <c r="A46" s="4">
         <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
@@ -3366,7 +3376,7 @@
       </c>
     </row>
     <row r="47" spans="1:11" s="6" customFormat="1">
-      <c r="A47" s="23">
+      <c r="A47" s="4">
         <v>46</v>
       </c>
       <c r="B47" s="4" t="s">
@@ -3399,7 +3409,7 @@
       </c>
     </row>
     <row r="48" spans="1:11" s="6" customFormat="1">
-      <c r="A48" s="23">
+      <c r="A48" s="4">
         <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
@@ -3432,7 +3442,7 @@
       </c>
     </row>
     <row r="49" spans="1:11" s="6" customFormat="1">
-      <c r="A49" s="23">
+      <c r="A49" s="4">
         <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
@@ -3465,7 +3475,7 @@
       </c>
     </row>
     <row r="50" spans="1:11" s="6" customFormat="1">
-      <c r="A50" s="23">
+      <c r="A50" s="4">
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
@@ -3497,7 +3507,7 @@
       </c>
     </row>
     <row r="51" spans="1:11" s="6" customFormat="1">
-      <c r="A51" s="23">
+      <c r="A51" s="4">
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
@@ -3529,7 +3539,7 @@
       </c>
     </row>
     <row r="52" spans="1:11" s="6" customFormat="1">
-      <c r="A52" s="23">
+      <c r="A52" s="4">
         <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
@@ -3562,7 +3572,7 @@
       </c>
     </row>
     <row r="53" spans="1:11" s="6" customFormat="1">
-      <c r="A53" s="23">
+      <c r="A53" s="4">
         <v>52</v>
       </c>
       <c r="B53" s="4" t="s">
@@ -3594,7 +3604,7 @@
       </c>
     </row>
     <row r="54" spans="1:11" s="6" customFormat="1">
-      <c r="A54" s="23">
+      <c r="A54" s="4">
         <v>53</v>
       </c>
       <c r="B54" s="4" t="s">
@@ -3626,7 +3636,7 @@
       </c>
     </row>
     <row r="55" spans="1:11" s="6" customFormat="1">
-      <c r="A55" s="23">
+      <c r="A55" s="4">
         <v>54</v>
       </c>
       <c r="B55" s="4" t="s">
@@ -3658,7 +3668,7 @@
       </c>
     </row>
     <row r="56" spans="1:11" s="6" customFormat="1">
-      <c r="A56" s="23">
+      <c r="A56" s="4">
         <v>55</v>
       </c>
       <c r="B56" s="4" t="s">
@@ -3690,7 +3700,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" s="6" customFormat="1">
-      <c r="A57" s="23">
+      <c r="A57" s="4">
         <v>56</v>
       </c>
       <c r="B57" s="4" t="s">
@@ -3722,7 +3732,7 @@
       </c>
     </row>
     <row r="58" spans="1:11" s="6" customFormat="1">
-      <c r="A58" s="23">
+      <c r="A58" s="4">
         <v>57</v>
       </c>
       <c r="B58" s="4" t="s">
@@ -3754,7 +3764,7 @@
       </c>
     </row>
     <row r="59" spans="1:11" s="6" customFormat="1">
-      <c r="A59" s="23">
+      <c r="A59" s="4">
         <v>58</v>
       </c>
       <c r="B59" s="4" t="s">
@@ -3786,7 +3796,7 @@
       </c>
     </row>
     <row r="60" spans="1:11" s="6" customFormat="1">
-      <c r="A60" s="23">
+      <c r="A60" s="4">
         <v>59</v>
       </c>
       <c r="B60" s="4" t="s">
@@ -3819,7 +3829,7 @@
       </c>
     </row>
     <row r="61" spans="1:11" s="6" customFormat="1">
-      <c r="A61" s="23">
+      <c r="A61" s="4">
         <v>60</v>
       </c>
       <c r="B61" s="4" t="s">
@@ -3852,7 +3862,7 @@
       </c>
     </row>
     <row r="62" spans="1:11" s="6" customFormat="1">
-      <c r="A62" s="23">
+      <c r="A62" s="4">
         <v>61</v>
       </c>
       <c r="B62" s="4" t="s">
@@ -3885,7 +3895,7 @@
       </c>
     </row>
     <row r="63" spans="1:11" s="6" customFormat="1">
-      <c r="A63" s="23">
+      <c r="A63" s="4">
         <v>62</v>
       </c>
       <c r="B63" s="4" t="s">
@@ -3918,7 +3928,7 @@
       </c>
     </row>
     <row r="64" spans="1:11" s="6" customFormat="1">
-      <c r="A64" s="23">
+      <c r="A64" s="4">
         <v>63</v>
       </c>
       <c r="B64" s="4" t="s">
@@ -3950,7 +3960,7 @@
       </c>
     </row>
     <row r="65" spans="1:11" s="6" customFormat="1">
-      <c r="A65" s="23">
+      <c r="A65" s="4">
         <v>64</v>
       </c>
       <c r="B65" s="4" t="s">
@@ -3982,7 +3992,7 @@
       </c>
     </row>
     <row r="66" spans="1:11" s="6" customFormat="1">
-      <c r="A66" s="23">
+      <c r="A66" s="4">
         <v>65</v>
       </c>
       <c r="B66" s="4" t="s">
@@ -4015,7 +4025,7 @@
       </c>
     </row>
     <row r="67" spans="1:11" s="6" customFormat="1">
-      <c r="A67" s="23">
+      <c r="A67" s="4">
         <v>66</v>
       </c>
       <c r="B67" s="4" t="s">
@@ -4048,7 +4058,7 @@
       </c>
     </row>
     <row r="68" spans="1:11" s="6" customFormat="1">
-      <c r="A68" s="23">
+      <c r="A68" s="4">
         <v>67</v>
       </c>
       <c r="B68" s="4" t="s">
@@ -4081,7 +4091,7 @@
       </c>
     </row>
     <row r="69" spans="1:11" s="6" customFormat="1">
-      <c r="A69" s="23">
+      <c r="A69" s="4">
         <v>68</v>
       </c>
       <c r="B69" s="4" t="s">
@@ -4114,7 +4124,7 @@
       </c>
     </row>
     <row r="70" spans="1:11" s="6" customFormat="1">
-      <c r="A70" s="23">
+      <c r="A70" s="4">
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
@@ -4147,7 +4157,7 @@
       </c>
     </row>
     <row r="71" spans="1:11" s="6" customFormat="1">
-      <c r="A71" s="23">
+      <c r="A71" s="4">
         <v>70</v>
       </c>
       <c r="B71" s="4" t="s">
@@ -4179,7 +4189,7 @@
       </c>
     </row>
     <row r="72" spans="1:11" s="6" customFormat="1">
-      <c r="A72" s="23">
+      <c r="A72" s="4">
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
@@ -4211,7 +4221,7 @@
       </c>
     </row>
     <row r="73" spans="1:11" s="6" customFormat="1">
-      <c r="A73" s="23">
+      <c r="A73" s="4">
         <v>72</v>
       </c>
       <c r="B73" s="4" t="s">
@@ -4243,7 +4253,7 @@
       </c>
     </row>
     <row r="74" spans="1:11" s="6" customFormat="1">
-      <c r="A74" s="23">
+      <c r="A74" s="4">
         <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
@@ -4275,7 +4285,7 @@
       </c>
     </row>
     <row r="75" spans="1:11" s="6" customFormat="1">
-      <c r="A75" s="23">
+      <c r="A75" s="4">
         <v>74</v>
       </c>
       <c r="B75" s="4" t="s">
@@ -4307,7 +4317,7 @@
       </c>
     </row>
     <row r="76" spans="1:11" s="6" customFormat="1">
-      <c r="A76" s="23">
+      <c r="A76" s="4">
         <v>75</v>
       </c>
       <c r="B76" s="4" t="s">
@@ -4340,7 +4350,7 @@
       </c>
     </row>
     <row r="77" spans="1:11" s="6" customFormat="1">
-      <c r="A77" s="23">
+      <c r="A77" s="4">
         <v>76</v>
       </c>
       <c r="B77" s="4" t="s">
@@ -4373,7 +4383,7 @@
       </c>
     </row>
     <row r="78" spans="1:11" s="6" customFormat="1">
-      <c r="A78" s="23">
+      <c r="A78" s="4">
         <v>77</v>
       </c>
       <c r="B78" s="4" t="s">
@@ -4406,7 +4416,7 @@
       </c>
     </row>
     <row r="79" spans="1:11" s="6" customFormat="1">
-      <c r="A79" s="23">
+      <c r="A79" s="4">
         <v>78</v>
       </c>
       <c r="B79" s="4" t="s">
@@ -4439,7 +4449,7 @@
       </c>
     </row>
     <row r="80" spans="1:11" s="6" customFormat="1">
-      <c r="A80" s="23">
+      <c r="A80" s="4">
         <v>79</v>
       </c>
       <c r="B80" s="4" t="s">
@@ -4471,7 +4481,7 @@
       </c>
     </row>
     <row r="81" spans="1:11" s="6" customFormat="1">
-      <c r="A81" s="23">
+      <c r="A81" s="4">
         <v>80</v>
       </c>
       <c r="B81" s="4" t="s">
@@ -4504,7 +4514,7 @@
       </c>
     </row>
     <row r="82" spans="1:11" s="6" customFormat="1">
-      <c r="A82" s="23">
+      <c r="A82" s="4">
         <v>81</v>
       </c>
       <c r="B82" s="4" t="s">
@@ -4537,7 +4547,7 @@
       </c>
     </row>
     <row r="83" spans="1:11" s="6" customFormat="1">
-      <c r="A83" s="23">
+      <c r="A83" s="4">
         <v>82</v>
       </c>
       <c r="B83" s="4" t="s">
@@ -4570,7 +4580,7 @@
       </c>
     </row>
     <row r="84" spans="1:11" s="6" customFormat="1">
-      <c r="A84" s="23">
+      <c r="A84" s="4">
         <v>83</v>
       </c>
       <c r="B84" s="4" t="s">
@@ -4602,7 +4612,7 @@
       </c>
     </row>
     <row r="85" spans="1:11" s="6" customFormat="1">
-      <c r="A85" s="23">
+      <c r="A85" s="4">
         <v>84</v>
       </c>
       <c r="B85" s="4" t="s">
@@ -4634,7 +4644,7 @@
       </c>
     </row>
     <row r="86" spans="1:11" s="6" customFormat="1">
-      <c r="A86" s="23">
+      <c r="A86" s="4">
         <v>85</v>
       </c>
       <c r="B86" s="4" t="s">
@@ -4665,7 +4675,7 @@
       </c>
     </row>
     <row r="87" spans="1:11" s="6" customFormat="1">
-      <c r="A87" s="23">
+      <c r="A87" s="4">
         <v>86</v>
       </c>
       <c r="B87" s="4" t="s">
@@ -4696,7 +4706,7 @@
       </c>
     </row>
     <row r="88" spans="1:11" s="6" customFormat="1">
-      <c r="A88" s="23">
+      <c r="A88" s="4">
         <v>87</v>
       </c>
       <c r="B88" s="4" t="s">
@@ -4727,7 +4737,7 @@
       </c>
     </row>
     <row r="89" spans="1:11" s="6" customFormat="1">
-      <c r="A89" s="23">
+      <c r="A89" s="4">
         <v>88</v>
       </c>
       <c r="B89" s="4" t="s">
@@ -4758,7 +4768,7 @@
       </c>
     </row>
     <row r="90" spans="1:11" s="6" customFormat="1">
-      <c r="A90" s="23">
+      <c r="A90" s="4">
         <v>89</v>
       </c>
       <c r="B90" s="4" t="s">
@@ -4789,7 +4799,7 @@
       </c>
     </row>
     <row r="91" spans="1:11" s="6" customFormat="1">
-      <c r="A91" s="23">
+      <c r="A91" s="4">
         <v>90</v>
       </c>
       <c r="B91" s="4" t="s">
@@ -4822,7 +4832,7 @@
       </c>
     </row>
     <row r="92" spans="1:11" s="6" customFormat="1">
-      <c r="A92" s="23">
+      <c r="A92" s="4">
         <v>91</v>
       </c>
       <c r="B92" s="4" t="s">
@@ -4855,7 +4865,7 @@
       </c>
     </row>
     <row r="93" spans="1:11" s="6" customFormat="1">
-      <c r="A93" s="23">
+      <c r="A93" s="4">
         <v>92</v>
       </c>
       <c r="B93" s="4" t="s">
@@ -4887,7 +4897,7 @@
       </c>
     </row>
     <row r="94" spans="1:11" s="6" customFormat="1">
-      <c r="A94" s="23">
+      <c r="A94" s="4">
         <v>93</v>
       </c>
       <c r="B94" s="4" t="s">
@@ -4919,7 +4929,7 @@
       </c>
     </row>
     <row r="95" spans="1:11" s="6" customFormat="1">
-      <c r="A95" s="23">
+      <c r="A95" s="4">
         <v>94</v>
       </c>
       <c r="B95" s="4" t="s">
@@ -4950,7 +4960,7 @@
       </c>
     </row>
     <row r="96" spans="1:11" s="6" customFormat="1">
-      <c r="A96" s="23">
+      <c r="A96" s="4">
         <v>95</v>
       </c>
       <c r="B96" s="4" t="s">
@@ -4983,7 +4993,7 @@
       </c>
     </row>
     <row r="97" spans="1:15" s="6" customFormat="1">
-      <c r="A97" s="23">
+      <c r="A97" s="4">
         <v>96</v>
       </c>
       <c r="B97" s="4" t="s">
@@ -5015,7 +5025,7 @@
       </c>
     </row>
     <row r="98" spans="1:15" s="6" customFormat="1">
-      <c r="A98" s="23">
+      <c r="A98" s="4">
         <v>97</v>
       </c>
       <c r="B98" s="4" t="s">
@@ -5047,7 +5057,7 @@
       </c>
     </row>
     <row r="99" spans="1:15" s="6" customFormat="1">
-      <c r="A99" s="23">
+      <c r="A99" s="4">
         <v>98</v>
       </c>
       <c r="B99" s="4" t="s">
@@ -5079,7 +5089,7 @@
       </c>
     </row>
     <row r="100" spans="1:15" s="6" customFormat="1">
-      <c r="A100" s="23">
+      <c r="A100" s="4">
         <v>99</v>
       </c>
       <c r="B100" s="4" t="s">
@@ -5112,7 +5122,7 @@
       </c>
     </row>
     <row r="101" spans="1:15" s="6" customFormat="1">
-      <c r="A101" s="23">
+      <c r="A101" s="4">
         <v>100</v>
       </c>
       <c r="B101" s="4" t="s">
@@ -5145,7 +5155,7 @@
       </c>
     </row>
     <row r="102" spans="1:15" s="6" customFormat="1">
-      <c r="A102" s="23">
+      <c r="A102" s="4">
         <v>101</v>
       </c>
       <c r="B102" s="4" t="s">
@@ -5176,7 +5186,7 @@
       </c>
     </row>
     <row r="103" spans="1:15" s="6" customFormat="1">
-      <c r="A103" s="23">
+      <c r="A103" s="4">
         <v>102</v>
       </c>
       <c r="B103" s="4" t="s">
@@ -5208,7 +5218,7 @@
       </c>
     </row>
     <row r="104" spans="1:15" s="6" customFormat="1">
-      <c r="A104" s="23">
+      <c r="A104" s="4">
         <v>103</v>
       </c>
       <c r="B104" s="4" t="s">
@@ -5240,7 +5250,7 @@
       </c>
     </row>
     <row r="105" spans="1:15" s="6" customFormat="1">
-      <c r="A105" s="23">
+      <c r="A105" s="4">
         <v>104</v>
       </c>
       <c r="B105" s="4" t="s">
@@ -5272,7 +5282,7 @@
       </c>
     </row>
     <row r="106" spans="1:15" s="6" customFormat="1">
-      <c r="A106" s="23">
+      <c r="A106" s="4">
         <v>105</v>
       </c>
       <c r="B106" s="4" t="s">
@@ -5304,7 +5314,7 @@
       </c>
     </row>
     <row r="107" spans="1:15" s="6" customFormat="1">
-      <c r="A107" s="23">
+      <c r="A107" s="4">
         <v>106</v>
       </c>
       <c r="B107" s="4" t="s">
@@ -5336,7 +5346,7 @@
       </c>
     </row>
     <row r="108" spans="1:15">
-      <c r="A108" s="23">
+      <c r="A108" s="4">
         <v>107</v>
       </c>
       <c r="B108" s="4" t="s">
@@ -5369,7 +5379,7 @@
       </c>
     </row>
     <row r="109" spans="1:15">
-      <c r="A109" s="23">
+      <c r="A109" s="4">
         <v>108</v>
       </c>
       <c r="B109" s="4" t="s">
@@ -5402,7 +5412,7 @@
       </c>
     </row>
     <row r="110" spans="1:15">
-      <c r="A110" s="23">
+      <c r="A110" s="4">
         <v>109</v>
       </c>
       <c r="B110" s="4" t="s">
@@ -5439,7 +5449,7 @@
       <c r="O110" s="6"/>
     </row>
     <row r="111" spans="1:15">
-      <c r="A111" s="23">
+      <c r="A111" s="4">
         <v>110</v>
       </c>
       <c r="B111" s="4" t="s">

</xml_diff>